<commit_message>
Update CUSTO PEÇAS IMPRESSAS.xlsx
</commit_message>
<xml_diff>
--- a/Impressao 3D/CUSTO PEÇAS IMPRESSAS.xlsx
+++ b/Impressao 3D/CUSTO PEÇAS IMPRESSAS.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Documents\Estudos\impressao-3D\Impressao 3D\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\REK\Documents\Estudos Claudio\impressao-3D\Impressao 3D\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -22,7 +22,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="2">Calculadora!$G$16</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">Impressão!$A$1:$E$29</definedName>
   </definedNames>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -390,10 +390,10 @@
     <t xml:space="preserve"> Valor Unidade</t>
   </si>
   <si>
-    <t>Chaveiro Kamila</t>
-  </si>
-  <si>
-    <t>SIM</t>
+    <t>Coelho Pascoa GR</t>
+  </si>
+  <si>
+    <t>NÃO</t>
   </si>
 </sst>
 </file>
@@ -417,11 +417,13 @@
       <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1715,19 +1717,19 @@
       </c>
       <c r="G4" s="19">
         <f t="shared" ref="G4:G9" si="0">$B$18*(1+F4/100)</f>
-        <v>13.67056</v>
+        <v>99.122349333333332</v>
       </c>
       <c r="H4" s="19">
         <f t="shared" ref="H4:H9" si="1">G4*E4</f>
-        <v>13.67056</v>
+        <v>99.122349333333332</v>
       </c>
       <c r="I4" s="19">
         <f t="shared" ref="I4:I9" si="2">G4-$B$18</f>
-        <v>10.25292</v>
+        <v>74.341762000000003</v>
       </c>
       <c r="J4" s="19">
         <f t="shared" ref="J4:J9" si="3">I4*E4</f>
-        <v>10.25292</v>
+        <v>74.341762000000003</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1745,19 +1747,19 @@
       </c>
       <c r="G5" s="19">
         <f t="shared" si="0"/>
-        <v>11.961740000000001</v>
+        <v>86.732055666666668</v>
       </c>
       <c r="H5" s="19">
         <f t="shared" si="1"/>
-        <v>59.808700000000002</v>
+        <v>433.66027833333334</v>
       </c>
       <c r="I5" s="19">
         <f t="shared" si="2"/>
-        <v>8.5441000000000003</v>
+        <v>61.951468333333338</v>
       </c>
       <c r="J5" s="19">
         <f t="shared" si="3"/>
-        <v>42.720500000000001</v>
+        <v>309.75734166666666</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1765,7 +1767,7 @@
         <v>58</v>
       </c>
       <c r="B6" s="23">
-        <v>18</v>
+        <v>191.46</v>
       </c>
       <c r="E6" s="3">
         <v>10</v>
@@ -1775,19 +1777,19 @@
       </c>
       <c r="G6" s="19">
         <f t="shared" si="0"/>
-        <v>10.25292</v>
+        <v>74.341762000000003</v>
       </c>
       <c r="H6" s="19">
         <f t="shared" si="1"/>
-        <v>102.5292</v>
+        <v>743.41762000000006</v>
       </c>
       <c r="I6" s="19">
         <f t="shared" si="2"/>
-        <v>6.8352799999999991</v>
+        <v>49.561174666666673</v>
       </c>
       <c r="J6" s="19">
         <f t="shared" si="3"/>
-        <v>68.352799999999988</v>
+        <v>495.6117466666667</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -1795,7 +1797,7 @@
         <v>59</v>
       </c>
       <c r="B7" s="23">
-        <v>1</v>
+        <v>5.8</v>
       </c>
       <c r="E7" s="3">
         <v>25</v>
@@ -1805,19 +1807,19 @@
       </c>
       <c r="G7" s="19">
         <f t="shared" si="0"/>
-        <v>8.5441000000000003</v>
+        <v>61.951468333333331</v>
       </c>
       <c r="H7" s="19">
         <f t="shared" si="1"/>
-        <v>213.60250000000002</v>
+        <v>1548.7867083333333</v>
       </c>
       <c r="I7" s="19">
         <f t="shared" si="2"/>
-        <v>5.1264599999999998</v>
+        <v>37.170880999999994</v>
       </c>
       <c r="J7" s="19">
         <f t="shared" si="3"/>
-        <v>128.16149999999999</v>
+        <v>929.27202499999987</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -1835,19 +1837,19 @@
       </c>
       <c r="G8" s="19">
         <f t="shared" si="0"/>
-        <v>7.5188080000000008</v>
+        <v>54.517292133333335</v>
       </c>
       <c r="H8" s="19">
         <f t="shared" si="1"/>
-        <v>375.94040000000007</v>
+        <v>2725.8646066666665</v>
       </c>
       <c r="I8" s="19">
         <f t="shared" si="2"/>
-        <v>4.1011680000000013</v>
+        <v>29.736704800000002</v>
       </c>
       <c r="J8" s="19">
         <f t="shared" si="3"/>
-        <v>205.05840000000006</v>
+        <v>1486.8352400000001</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1865,19 +1867,19 @@
       </c>
       <c r="G9" s="19">
         <f t="shared" si="0"/>
-        <v>6.83528</v>
+        <v>49.561174666666666</v>
       </c>
       <c r="H9" s="19">
         <f t="shared" si="1"/>
-        <v>683.52800000000002</v>
+        <v>4956.1174666666666</v>
       </c>
       <c r="I9" s="19">
         <f t="shared" si="2"/>
-        <v>3.41764</v>
+        <v>24.780587333333333</v>
       </c>
       <c r="J9" s="19">
         <f t="shared" si="3"/>
-        <v>341.76400000000001</v>
+        <v>2478.0587333333333</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -1895,19 +1897,19 @@
       </c>
       <c r="G10" s="19">
         <f>$B$18*(1+F10/100)</f>
-        <v>6.1517520000000001</v>
+        <v>44.605057199999997</v>
       </c>
       <c r="H10" s="19">
         <f>G10*E10</f>
-        <v>3075.8760000000002</v>
+        <v>22302.528599999998</v>
       </c>
       <c r="I10" s="19">
         <f>G10-$B$18</f>
-        <v>2.7341120000000001</v>
+        <v>19.824469866666664</v>
       </c>
       <c r="J10" s="19">
         <f>I10*E10</f>
-        <v>1367.056</v>
+        <v>9912.2349333333314</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -1919,19 +1921,19 @@
       </c>
       <c r="G11" s="19">
         <f>$B$18*(1+F11/100)</f>
-        <v>5.8099879999999997</v>
+        <v>42.126998466666663</v>
       </c>
       <c r="H11" s="19">
         <f>G11*E11</f>
-        <v>5809.9879999999994</v>
+        <v>42126.998466666664</v>
       </c>
       <c r="I11" s="19">
         <f>G11-$B$18</f>
-        <v>2.3923479999999997</v>
+        <v>17.34641113333333</v>
       </c>
       <c r="J11" s="19">
         <f>I11*E11</f>
-        <v>2392.3479999999995</v>
+        <v>17346.411133333331</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -1949,19 +1951,19 @@
       </c>
       <c r="G12" s="19">
         <f>$B$18*(1+F12/100)</f>
-        <v>5.4682240000000002</v>
+        <v>39.648939733333336</v>
       </c>
       <c r="H12" s="19">
         <f>G12*E12</f>
-        <v>13670.560000000001</v>
+        <v>99122.349333333346</v>
       </c>
       <c r="I12" s="19">
         <f>G12-$B$18</f>
-        <v>2.0505840000000002</v>
+        <v>14.868352400000003</v>
       </c>
       <c r="J12" s="19">
         <f>I12*E12</f>
-        <v>5126.46</v>
+        <v>37170.881000000008</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -1970,7 +1972,7 @@
       </c>
       <c r="B13" s="38">
         <f>B6/1000*VLOOKUP(B5,Configurações!$A$7:$B$11,2,FALSE)</f>
-        <v>1.7081999999999999</v>
+        <v>18.169554000000002</v>
       </c>
       <c r="E13" s="36"/>
       <c r="F13" s="36"/>
@@ -1985,7 +1987,7 @@
       </c>
       <c r="B14" s="38">
         <f>B7*0.25*Configurações!$B$4</f>
-        <v>0.3</v>
+        <v>1.74</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1994,7 +1996,7 @@
       </c>
       <c r="B15" s="38">
         <f>VLOOKUP(B8,Configurações!$A$14:$B$22,2,FALSE)/(Configurações!$B$26*Configurações!$B$27)*B7</f>
-        <v>0.83983333333333332</v>
+        <v>4.8710333333333331</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -2005,7 +2007,7 @@
       </c>
       <c r="B16" s="38">
         <f>B13+B14+B15</f>
-        <v>2.8480333333333334</v>
+        <v>24.780587333333333</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -2014,7 +2016,7 @@
       </c>
       <c r="B17" s="38">
         <f>IF(B9="SIM",B16*(1+Configurações!$B$33/100),B16)</f>
-        <v>3.41764</v>
+        <v>24.780587333333333</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -2023,7 +2025,7 @@
       </c>
       <c r="B18" s="38">
         <f>B17</f>
-        <v>3.41764</v>
+        <v>24.780587333333333</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -2038,7 +2040,7 @@
       </c>
       <c r="J20" s="13">
         <f>B18*Configurações!$B$30/100</f>
-        <v>0.68352800000000002</v>
+        <v>4.9561174666666661</v>
       </c>
     </row>
   </sheetData>
@@ -2092,7 +2094,7 @@
     <row r="9" spans="2:4" ht="15.75" thickBot="1">
       <c r="B9" s="41" t="str">
         <f>Calculadora!B4</f>
-        <v>Chaveiro Kamila</v>
+        <v>Coelho Pascoa GR</v>
       </c>
       <c r="C9" s="42"/>
       <c r="D9" s="43"/>
@@ -2125,7 +2127,7 @@
       </c>
       <c r="C13" s="27">
         <f>Calculadora!G4</f>
-        <v>13.67056</v>
+        <v>99.122349333333332</v>
       </c>
       <c r="D13" s="39">
         <f>ROUNDUP((Calculadora!B7+12)/24,0)</f>
@@ -2139,11 +2141,11 @@
       </c>
       <c r="C14" s="26">
         <f>Calculadora!G5</f>
-        <v>11.961740000000001</v>
+        <v>86.732055666666668</v>
       </c>
       <c r="D14" s="40">
         <f>ROUNDUP(((Calculadora!B7*B14+12)/Calculadora!B10)/24,0)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="2:4">
@@ -2153,11 +2155,11 @@
       </c>
       <c r="C15" s="27">
         <f>Calculadora!G6</f>
-        <v>10.25292</v>
+        <v>74.341762000000003</v>
       </c>
       <c r="D15" s="39">
         <f>ROUNDUP((Calculadora!B7*B15+12)/Calculadora!B10/24,0)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="2:4">
@@ -2167,11 +2169,11 @@
       </c>
       <c r="C16" s="26">
         <f>Calculadora!G7</f>
-        <v>8.5441000000000003</v>
+        <v>61.951468333333331</v>
       </c>
       <c r="D16" s="40">
         <f>ROUNDUP((Calculadora!B7*B16+12)/Calculadora!B10/24,0)</f>
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="2:4">
@@ -2181,11 +2183,11 @@
       </c>
       <c r="C17" s="27">
         <f>Calculadora!G8</f>
-        <v>7.5188080000000008</v>
+        <v>54.517292133333335</v>
       </c>
       <c r="D17" s="39">
         <f>ROUNDUP((Calculadora!B7*B17+12)/Calculadora!B10/24,0)</f>
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="2:4">
@@ -2195,11 +2197,11 @@
       </c>
       <c r="C18" s="26">
         <f>Calculadora!G9</f>
-        <v>6.83528</v>
+        <v>49.561174666666666</v>
       </c>
       <c r="D18" s="40">
         <f>ROUNDUP((Calculadora!B7*B18+12)/Calculadora!B10/24,0)</f>
-        <v>5</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="2:4">
@@ -2209,11 +2211,11 @@
       </c>
       <c r="C19" s="27">
         <f>Calculadora!G10</f>
-        <v>6.1517520000000001</v>
+        <v>44.605057199999997</v>
       </c>
       <c r="D19" s="39">
         <f>ROUNDUP((Calculadora!B7*B19+12)/Calculadora!B10/24,0)</f>
-        <v>22</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="2:4">
@@ -2223,11 +2225,11 @@
       </c>
       <c r="C20" s="26">
         <f>Calculadora!G11</f>
-        <v>5.8099879999999997</v>
+        <v>42.126998466666663</v>
       </c>
       <c r="D20" s="40">
         <f>ROUNDUP((Calculadora!B7*B20+12)/Calculadora!B10/24,0)</f>
-        <v>43</v>
+        <v>243</v>
       </c>
     </row>
     <row r="21" spans="2:4">
@@ -2237,11 +2239,11 @@
       </c>
       <c r="C21" s="27">
         <f>Calculadora!G12</f>
-        <v>5.4682240000000002</v>
+        <v>39.648939733333336</v>
       </c>
       <c r="D21" s="39">
         <f>ROUNDUP((Calculadora!B7*B21+12)/Calculadora!B10/24,0)</f>
-        <v>105</v>
+        <v>605</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Create ~$CUSTO PEÇAS IMPRESSAS.xlsx
</commit_message>
<xml_diff>
--- a/Impressao 3D/CUSTO PEÇAS IMPRESSAS.xlsx
+++ b/Impressao 3D/CUSTO PEÇAS IMPRESSAS.xlsx
@@ -1717,19 +1717,19 @@
       </c>
       <c r="G4" s="19">
         <f t="shared" ref="G4:G9" si="0">$B$18*(1+F4/100)</f>
-        <v>72.948933333333329</v>
+        <v>109.16733333333333</v>
       </c>
       <c r="H4" s="19">
         <f t="shared" ref="H4:H9" si="1">G4*E4</f>
-        <v>72.948933333333329</v>
+        <v>109.16733333333333</v>
       </c>
       <c r="I4" s="19">
         <f t="shared" ref="I4:I9" si="2">G4-$B$18</f>
-        <v>54.711699999999993</v>
+        <v>81.875500000000002</v>
       </c>
       <c r="J4" s="19">
         <f t="shared" ref="J4:J9" si="3">I4*E4</f>
-        <v>54.711699999999993</v>
+        <v>81.875500000000002</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1747,19 +1747,19 @@
       </c>
       <c r="G5" s="19">
         <f t="shared" si="0"/>
-        <v>63.830316666666661</v>
+        <v>95.521416666666667</v>
       </c>
       <c r="H5" s="19">
         <f t="shared" si="1"/>
-        <v>319.15158333333329</v>
+        <v>477.60708333333332</v>
       </c>
       <c r="I5" s="19">
         <f t="shared" si="2"/>
-        <v>45.593083333333325</v>
+        <v>68.229583333333338</v>
       </c>
       <c r="J5" s="19">
         <f t="shared" si="3"/>
-        <v>227.96541666666661</v>
+        <v>341.14791666666667</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1767,7 +1767,7 @@
         <v>58</v>
       </c>
       <c r="B6" s="23">
-        <v>146</v>
+        <v>217</v>
       </c>
       <c r="E6" s="3">
         <v>10</v>
@@ -1777,19 +1777,19 @@
       </c>
       <c r="G6" s="19">
         <f t="shared" si="0"/>
-        <v>54.711699999999993</v>
+        <v>81.875500000000002</v>
       </c>
       <c r="H6" s="19">
         <f t="shared" si="1"/>
-        <v>547.11699999999996</v>
+        <v>818.755</v>
       </c>
       <c r="I6" s="19">
         <f t="shared" si="2"/>
-        <v>36.474466666666657</v>
+        <v>54.583666666666673</v>
       </c>
       <c r="J6" s="19">
         <f t="shared" si="3"/>
-        <v>364.7446666666666</v>
+        <v>545.8366666666667</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -1797,7 +1797,7 @@
         <v>59</v>
       </c>
       <c r="B7" s="23">
-        <v>4.5999999999999996</v>
+        <v>7</v>
       </c>
       <c r="E7" s="3">
         <v>25</v>
@@ -1807,19 +1807,19 @@
       </c>
       <c r="G7" s="19">
         <f t="shared" si="0"/>
-        <v>45.593083333333333</v>
+        <v>68.229583333333338</v>
       </c>
       <c r="H7" s="19">
         <f t="shared" si="1"/>
-        <v>1139.8270833333333</v>
+        <v>1705.7395833333335</v>
       </c>
       <c r="I7" s="19">
         <f t="shared" si="2"/>
-        <v>27.35585</v>
+        <v>40.937750000000008</v>
       </c>
       <c r="J7" s="19">
         <f t="shared" si="3"/>
-        <v>683.89625000000001</v>
+        <v>1023.4437500000003</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -1837,19 +1837,19 @@
       </c>
       <c r="G8" s="19">
         <f t="shared" si="0"/>
-        <v>40.121913333333332</v>
+        <v>60.042033333333336</v>
       </c>
       <c r="H8" s="19">
         <f t="shared" si="1"/>
-        <v>2006.0956666666666</v>
+        <v>3002.1016666666669</v>
       </c>
       <c r="I8" s="19">
         <f t="shared" si="2"/>
-        <v>21.884679999999999</v>
+        <v>32.750200000000007</v>
       </c>
       <c r="J8" s="19">
         <f t="shared" si="3"/>
-        <v>1094.2339999999999</v>
+        <v>1637.5100000000002</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -1867,19 +1867,19 @@
       </c>
       <c r="G9" s="19">
         <f t="shared" si="0"/>
-        <v>36.474466666666665</v>
+        <v>54.583666666666666</v>
       </c>
       <c r="H9" s="19">
         <f t="shared" si="1"/>
-        <v>3647.4466666666663</v>
+        <v>5458.3666666666668</v>
       </c>
       <c r="I9" s="19">
         <f t="shared" si="2"/>
-        <v>18.237233333333332</v>
+        <v>27.291833333333333</v>
       </c>
       <c r="J9" s="19">
         <f t="shared" si="3"/>
-        <v>1823.7233333333331</v>
+        <v>2729.1833333333334</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -1897,19 +1897,19 @@
       </c>
       <c r="G10" s="19">
         <f>$B$18*(1+F10/100)</f>
-        <v>32.827019999999997</v>
+        <v>49.125300000000003</v>
       </c>
       <c r="H10" s="19">
         <f>G10*E10</f>
-        <v>16413.509999999998</v>
+        <v>24562.65</v>
       </c>
       <c r="I10" s="19">
         <f>G10-$B$18</f>
-        <v>14.589786666666665</v>
+        <v>21.83346666666667</v>
       </c>
       <c r="J10" s="19">
         <f>I10*E10</f>
-        <v>7294.8933333333325</v>
+        <v>10916.733333333335</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -1921,19 +1921,19 @@
       </c>
       <c r="G11" s="19">
         <f>$B$18*(1+F11/100)</f>
-        <v>31.003296666666664</v>
+        <v>46.396116666666664</v>
       </c>
       <c r="H11" s="19">
         <f>G11*E11</f>
-        <v>31003.296666666665</v>
+        <v>46396.116666666661</v>
       </c>
       <c r="I11" s="19">
         <f>G11-$B$18</f>
-        <v>12.766063333333332</v>
+        <v>19.104283333333331</v>
       </c>
       <c r="J11" s="19">
         <f>I11*E11</f>
-        <v>12766.063333333332</v>
+        <v>19104.283333333333</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -1951,19 +1951,19 @@
       </c>
       <c r="G12" s="19">
         <f>$B$18*(1+F12/100)</f>
-        <v>29.179573333333334</v>
+        <v>43.666933333333333</v>
       </c>
       <c r="H12" s="19">
         <f>G12*E12</f>
-        <v>72948.933333333334</v>
+        <v>109167.33333333333</v>
       </c>
       <c r="I12" s="19">
         <f>G12-$B$18</f>
-        <v>10.942340000000002</v>
+        <v>16.3751</v>
       </c>
       <c r="J12" s="19">
         <f>I12*E12</f>
-        <v>27355.850000000002</v>
+        <v>40937.75</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="B13" s="38">
         <f>B6/1000*VLOOKUP(B5,Configurações!$A$7:$B$11,2,FALSE)</f>
-        <v>12.994</v>
+        <v>19.312999999999999</v>
       </c>
       <c r="E13" s="36"/>
       <c r="F13" s="36"/>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="B14" s="38">
         <f>B7*0.25*Configurações!$B$4</f>
-        <v>1.38</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="B15" s="38">
         <f>VLOOKUP(B8,Configurações!$A$14:$B$22,2,FALSE)/(Configurações!$B$26*Configurações!$B$27)*B7</f>
-        <v>3.8632333333333331</v>
+        <v>5.8788333333333336</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="B16" s="38">
         <f>B13+B14+B15</f>
-        <v>18.237233333333332</v>
+        <v>27.291833333333333</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B17" s="38">
         <f>IF(B9="SIM",B16*(1+Configurações!$B$33/100),B16)</f>
-        <v>18.237233333333332</v>
+        <v>27.291833333333333</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="B18" s="38">
         <f>B17</f>
-        <v>18.237233333333332</v>
+        <v>27.291833333333333</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="J20" s="13">
         <f>B18*Configurações!$B$30/100</f>
-        <v>3.6474466666666667</v>
+        <v>5.4583666666666666</v>
       </c>
     </row>
   </sheetData>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="C13" s="27">
         <f>Calculadora!G4</f>
-        <v>72.948933333333329</v>
+        <v>109.16733333333333</v>
       </c>
       <c r="D13" s="39">
         <f>ROUNDUP((Calculadora!B7+12)/24,0)</f>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="C14" s="26">
         <f>Calculadora!G5</f>
-        <v>63.830316666666661</v>
+        <v>95.521416666666667</v>
       </c>
       <c r="D14" s="40">
         <f>ROUNDUP(((Calculadora!B7*B14+12)/Calculadora!B10)/24,0)</f>
@@ -2155,11 +2155,11 @@
       </c>
       <c r="C15" s="27">
         <f>Calculadora!G6</f>
-        <v>54.711699999999993</v>
+        <v>81.875500000000002</v>
       </c>
       <c r="D15" s="39">
         <f>ROUNDUP((Calculadora!B7*B15+12)/Calculadora!B10/24,0)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="2:4">
@@ -2169,11 +2169,11 @@
       </c>
       <c r="C16" s="26">
         <f>Calculadora!G7</f>
-        <v>45.593083333333333</v>
+        <v>68.229583333333338</v>
       </c>
       <c r="D16" s="40">
         <f>ROUNDUP((Calculadora!B7*B16+12)/Calculadora!B10/24,0)</f>
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17" spans="2:4">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C17" s="27">
         <f>Calculadora!G8</f>
-        <v>40.121913333333332</v>
+        <v>60.042033333333336</v>
       </c>
       <c r="D17" s="39">
         <f>ROUNDUP((Calculadora!B7*B17+12)/Calculadora!B10/24,0)</f>
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" spans="2:4">
@@ -2197,11 +2197,11 @@
       </c>
       <c r="C18" s="26">
         <f>Calculadora!G9</f>
-        <v>36.474466666666665</v>
+        <v>54.583666666666666</v>
       </c>
       <c r="D18" s="40">
         <f>ROUNDUP((Calculadora!B7*B18+12)/Calculadora!B10/24,0)</f>
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="2:4">
@@ -2211,11 +2211,11 @@
       </c>
       <c r="C19" s="27">
         <f>Calculadora!G10</f>
-        <v>32.827019999999997</v>
+        <v>49.125300000000003</v>
       </c>
       <c r="D19" s="39">
         <f>ROUNDUP((Calculadora!B7*B19+12)/Calculadora!B10/24,0)</f>
-        <v>97</v>
+        <v>147</v>
       </c>
     </row>
     <row r="20" spans="2:4">
@@ -2225,11 +2225,11 @@
       </c>
       <c r="C20" s="26">
         <f>Calculadora!G11</f>
-        <v>31.003296666666664</v>
+        <v>46.396116666666664</v>
       </c>
       <c r="D20" s="40">
         <f>ROUNDUP((Calculadora!B7*B20+12)/Calculadora!B10/24,0)</f>
-        <v>193</v>
+        <v>293</v>
       </c>
     </row>
     <row r="21" spans="2:4">
@@ -2239,11 +2239,11 @@
       </c>
       <c r="C21" s="27">
         <f>Calculadora!G12</f>
-        <v>29.179573333333334</v>
+        <v>43.666933333333333</v>
       </c>
       <c r="D21" s="39">
         <f>ROUNDUP((Calculadora!B7*B21+12)/Calculadora!B10/24,0)</f>
-        <v>480</v>
+        <v>730</v>
       </c>
     </row>
   </sheetData>

</xml_diff>